<commit_message>
chore: remove the startup banner from all three projects
It did its job. The MH.RevitTools rename is confirmed working, and a modal
dialog on every Revit start is not something to leave in.

All three App.cs files are byte-identical to their state before e825f8d, so
this is a clean revert of the marker and nothing else. Verified 2026 and 2027
still build.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Revit.Addin.2024/version-docs.xlsx
+++ b/Revit.Addin.2024/version-docs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Y.Abdelazziz\source\repos\Revit2024\Revit.Addin.2024\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Y.Abdelazziz\source\repos\Revit.Addin.MultiVersion\Revit.Addin.2024\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{041E40E8-D0FB-4A33-BF62-6618F69A568D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB3C400-1545-493D-906A-24E7E5A7A802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="960" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="79">
   <si>
     <t>Version</t>
   </si>
@@ -253,6 +253,15 @@
   </si>
   <si>
     <t xml:space="preserve">Familyupdater feature updated </t>
+  </si>
+  <si>
+    <t>5.1.1.0</t>
+  </si>
+  <si>
+    <t>Routine update.</t>
+  </si>
+  <si>
+    <t>5.1.2.0</t>
   </si>
 </sst>
 </file>
@@ -601,7 +610,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.88671875" customWidth="1"/>
@@ -910,6 +919,22 @@
       </c>
       <c r="B38" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>76</v>
+      </c>
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>78</v>
+      </c>
+      <c r="B40" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>